<commit_message>
Add Deepgram Nova-3, MSDD telephonic, and Nemotron 3.5 pipeline diarization
</commit_message>
<xml_diff>
--- a/Diarization-models.xlsx
+++ b/Diarization-models.xlsx
@@ -103,6 +103,9 @@
     <xf numFmtId="165" fontId="2" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf fontId="2" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -115,13 +118,14 @@
   <dimension ref="A1:P50"/>
   <cols>
     <col min="1" max="1" width="41.67832167832167" style="1"/>
-    <col min="2" max="2" width="6.8531468531468525" style="1"/>
+    <col min="2" max="2" width="6.153846153846153" style="1"/>
     <col min="3" max="3" width="26.433566433566433" style="1"/>
     <col min="4" max="4" width="17.62237762237762" style="1"/>
     <col min="5" max="5" width="24.895104895104893" style="1"/>
     <col min="6" max="6" width="20.41958041958042" style="1"/>
     <col min="7" max="7" width="23.496503496503497" style="1"/>
-    <col min="8" max="9" width="13.986013986013985" style="1"/>
+    <col min="8" max="8" width="20.41958041958042" style="1"/>
+    <col min="9" max="9" width="14.965034965034965" style="1"/>
     <col min="10" max="16" width="13.986013986013985" style="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -148,6 +152,9 @@
         <v>talkbank/callhome DER
 (Locally 5 files only)</v>
       </c>
+      <c r="H1" s="2" t="str">
+        <v>Cost</v>
+      </c>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -175,9 +182,11 @@
       <c r="G2" s="9">
         <v>0.2069</v>
       </c>
-      <c r="H2" s="5"/>
-    </row>
-    <row r="3">
+      <c r="H2" s="7" t="str">
+        <v>local </v>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="4" t="str">
         <v>Pyannote speaker-diarization-community-1</v>
       </c>
@@ -200,7 +209,10 @@
       <c r="G3" s="9">
         <v>0.2057</v>
       </c>
-      <c r="H3" s="5"/>
+      <c r="H3" s="10" t="str">
+        <v>Local also available
+~€0.00058/min(API)</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="str">
@@ -210,7 +222,7 @@
         <v>API</v>
       </c>
       <c r="C4" s="5" t="str">
-        <v>Commercial</v>
+        <v>Commercial API</v>
       </c>
       <c r="D4" s="7" t="str">
         <v>Not published</v>
@@ -224,7 +236,9 @@
       <c r="G4" s="9">
         <v>0.1165</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="7" t="str">
+        <v>~€0.0016/min</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
@@ -234,7 +248,7 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
-      <c r="H5" s="5"/>
+      <c r="H5" s="7"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="str">
@@ -259,7 +273,9 @@
       <c r="G6" s="9">
         <v>0.1745</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="H6" s="7" t="str">
+        <v>local</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="str">
@@ -283,7 +299,9 @@
       <c r="G7" s="9">
         <v>0.1536</v>
       </c>
-      <c r="H7" s="5"/>
+      <c r="H7" s="7" t="str">
+        <v>local</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="str">
@@ -308,47 +326,81 @@
       <c r="G8" s="9">
         <v>0.1404</v>
       </c>
-      <c r="H8" s="5"/>
+      <c r="H8" s="7" t="str">
+        <v>local</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="5"/>
+      <c r="A9" s="4" t="str">
+        <v>Nvidia Diarization MSDD Telephonic</v>
+      </c>
+      <c r="B9" s="5" t="str">
+        <v>OSS</v>
+      </c>
+      <c r="C9" s="5" t="str">
+        <v>NGC TERMS OF USE</v>
+      </c>
+      <c r="D9" s="7" t="str">
+        <v>~31.1M</v>
+      </c>
+      <c r="E9" s="7" t="str">
+        <v>Not published</v>
+      </c>
+      <c r="F9" s="7" t="str">
+        <v>Not published</v>
+      </c>
+      <c r="G9" s="7" t="str">
+        <v>N/A (benchmark failed)</v>
+      </c>
+      <c r="H9" s="7" t="str">
+        <v>local</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="A11" s="4" t="str">
+        <v>Deepgram nova-3-diarize-v2</v>
+      </c>
+      <c r="B11" s="5" t="str">
+        <v>API</v>
+      </c>
+      <c r="C11" s="5" t="str">
+        <v>Commercial API</v>
+      </c>
+      <c r="D11" s="7" t="str">
+        <v>Not published</v>
+      </c>
+      <c r="E11" s="7" t="str">
+        <v>Not published</v>
+      </c>
+      <c r="F11" s="7" t="str">
+        <v>Not published</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.33880000000000005</v>
+      </c>
+      <c r="H11" s="7" t="str">
+        <v>~$0.0052/min</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
     </row>
     <row r="13">
       <c r="A13" s="5"/>

</xml_diff>